<commit_message>
ran tentative first trial
</commit_message>
<xml_diff>
--- a/test_cases/test_case_simplified.xlsx
+++ b/test_cases/test_case_simplified.xlsx
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="177" uniqueCount="94">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="178" uniqueCount="95">
   <si>
     <t>uid</t>
   </si>
@@ -78,6 +78,9 @@
   </si>
   <si>
     <t>Sn</t>
+  </si>
+  <si>
+    <t>pmax</t>
   </si>
   <si>
     <t>bus1</t>
@@ -1908,13 +1911,13 @@
 
 <file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1:O2"/>
+  <dimension ref="A1:P2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
     <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -1931,48 +1934,48 @@
         <v>13</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G1" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="H1" s="2" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="I1" s="2" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="J1" s="2" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="K1" s="2" t="s">
         <v>18</v>
       </c>
       <c r="L1" s="2" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="M1" s="2" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="N1" s="2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="O1" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
-    <row r="2" spans="1:15" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:16" x14ac:dyDescent="0.25">
       <c r="A2" s="2">
         <v>0</v>
       </c>
-      <c r="B2" s="2" t="s">
-        <v>92</v>
+      <c r="B2" s="2">
+        <v>1</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -1981,7 +1984,7 @@
         <v>1</v>
       </c>
       <c r="G2" s="2">
-        <v>0.15</v>
+        <v>10</v>
       </c>
       <c r="H2" s="2">
         <v>0.11</v>
@@ -2019,7 +2022,7 @@
   <dimension ref="A1:D2"/>
   <sheetFormatPr defaultRowHeight="15" outlineLevelRow="0" outlineLevelCol="0" x14ac:dyDescent="55"/>
   <cols>
-    <col min="1" max="28" width="13.571428571428571" customWidth="1"/>
+    <col min="1" max="24" width="13.571428571428571" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
@@ -2038,13 +2041,13 @@
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="B2">
         <v>1</v>
       </c>
       <c r="C2" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="D2">
         <v>1</v>
@@ -3223,8 +3226,12 @@
       <c r="G1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="H1" s="1"/>
-      <c r="I1" s="1"/>
+      <c r="H1" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>19</v>
+      </c>
       <c r="J1" s="1"/>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -3236,7 +3243,7 @@
       <c r="R1" s="1"/>
       <c r="S1" s="1"/>
     </row>
-    <row r="2" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A2" s="1">
         <v>0</v>
       </c>
@@ -3258,8 +3265,14 @@
       <c r="G2" s="2">
         <v>1</v>
       </c>
+      <c r="H2">
+        <v>0.4</v>
+      </c>
+      <c r="I2">
+        <v>999</v>
+      </c>
     </row>
-    <row r="3" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A3" s="1">
         <v>1</v>
       </c>
@@ -3281,8 +3294,14 @@
       <c r="G3" s="2">
         <v>2</v>
       </c>
+      <c r="H3">
+        <v>0.2</v>
+      </c>
+      <c r="I3">
+        <v>999</v>
+      </c>
     </row>
-    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A4" s="1">
         <v>2</v>
       </c>
@@ -3304,8 +3323,14 @@
       <c r="G4" s="2">
         <v>3</v>
       </c>
+      <c r="H4">
+        <v>0.2</v>
+      </c>
+      <c r="I4">
+        <v>999</v>
+      </c>
     </row>
-    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5">
         <v>0</v>
@@ -3324,6 +3349,12 @@
       </c>
       <c r="G5">
         <v>0</v>
+      </c>
+      <c r="H5">
+        <v>0</v>
+      </c>
+      <c r="I5">
+        <v>999</v>
       </c>
     </row>
     <row r="21" ht="15.75" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -4334,64 +4365,64 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="G1" s="1" t="s">
         <v>18</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
     </row>
     <row r="2" spans="1:21" x14ac:dyDescent="0.25">
@@ -4399,13 +4430,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -4464,13 +4495,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
@@ -4529,13 +4560,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>
@@ -4592,13 +4623,13 @@
     <row r="5" spans="1:17" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
       <c r="B5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="C5">
         <v>1</v>
       </c>
       <c r="D5" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E5">
         <v>0</v>
@@ -5722,13 +5753,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="C2" s="4">
         <v>1</v>
       </c>
       <c r="D2" s="4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E2" s="4">
         <v>100</v>
@@ -6026,10 +6057,10 @@
         <v>13</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="H1" s="1" t="s">
         <v>18</v>
@@ -6038,13 +6069,13 @@
         <v>4</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -6068,13 +6099,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E2" s="2">
         <v>2</v>
@@ -6095,7 +6126,7 @@
         <v>0</v>
       </c>
       <c r="L2" s="2">
-        <v>7.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="3" spans="1:12" x14ac:dyDescent="0.25">
@@ -6103,13 +6134,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E3" s="2">
         <v>3</v>
@@ -6130,7 +6161,7 @@
         <v>0</v>
       </c>
       <c r="L3" s="2">
-        <v>7.4</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4" spans="1:1" x14ac:dyDescent="0.25">
@@ -7151,22 +7182,22 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="K1" s="1"/>
       <c r="L1" s="1"/>
@@ -7178,16 +7209,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2">
         <v>200</v>
@@ -7210,16 +7241,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" s="2">
         <v>100</v>
@@ -8254,70 +8285,70 @@
         <v>3</v>
       </c>
       <c r="E1" s="1" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="J1" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="K1" s="1" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="L1" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="M1" s="1" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="N1" s="1" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="O1" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="P1" s="1" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="Q1" s="1" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="R1" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="S1" s="1" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="T1" s="1" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="U1" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="V1" s="1" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="W1" s="1" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="X1" s="1" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="Y1" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="Z1" s="1" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
     </row>
     <row r="2" spans="1:26" x14ac:dyDescent="0.25">
@@ -8325,16 +8356,16 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E2" s="2" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="F2" s="2">
         <v>0.02</v>
@@ -8405,16 +8436,16 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E3" s="2" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="F3" s="2">
         <v>0.02</v>
@@ -9498,13 +9529,13 @@
         <v>13</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>21</v>
+        <v>22</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
@@ -9512,13 +9543,13 @@
         <v>0</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="C2" s="2">
         <v>1</v>
       </c>
       <c r="D2" s="2" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E2" s="2">
         <v>1</v>
@@ -9538,13 +9569,13 @@
         <v>1</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="C3" s="2">
         <v>1</v>
       </c>
       <c r="D3" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E3" s="2">
         <v>2</v>
@@ -9564,13 +9595,13 @@
         <v>2</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C4" s="2">
         <v>1</v>
       </c>
       <c r="D4" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E4" s="2">
         <v>3</v>

</xml_diff>